<commit_message>
feat: generar comparativa cruda lado a lado con formato estandarizado
</commit_message>
<xml_diff>
--- a/eval_nlp/megadapt_evaluacion.xlsx
+++ b/eval_nlp/megadapt_evaluacion.xlsx
@@ -578,19 +578,19 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>0.7446</v>
+        <v>0.7764</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>0.7055</v>
+        <v>0.7671</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.7365</v>
+        <v>0.7725</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.7151</v>
+        <v>0.7231</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.7254</v>
+        <v>0.7598</v>
       </c>
     </row>
   </sheetData>
@@ -751,22 +751,22 @@
         <v>0.09329999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1805</v>
+        <v>0.1796</v>
       </c>
       <c r="J2" t="n">
         <v>0.2459</v>
       </c>
       <c r="K2" s="9" t="n">
-        <v>0.2082</v>
+        <v>0.2076</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7479</v>
+        <v>0.7482</v>
       </c>
       <c r="M2" t="n">
         <v>0.7936</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>0.7701</v>
+        <v>0.7702</v>
       </c>
     </row>
     <row r="3">
@@ -801,22 +801,22 @@
         <v>0.0455</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1908</v>
+        <v>0.1903</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2289</v>
+        <v>0.2249</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>0.2081</v>
+        <v>0.2062</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7402</v>
+        <v>0.7361</v>
       </c>
       <c r="M3" t="n">
         <v>0.7655999999999999</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>0.7527</v>
+        <v>0.7506</v>
       </c>
     </row>
     <row r="4">
@@ -842,31 +842,31 @@
         <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0472</v>
+        <v>0.0325</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0472</v>
+        <v>0.0325</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>0.0472</v>
+        <v>0.0325</v>
       </c>
       <c r="I4" t="n">
-        <v>0.179</v>
+        <v>0.1594</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1713</v>
+        <v>0.1518</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>0.1751</v>
+        <v>0.1555</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7739</v>
+        <v>0.7605</v>
       </c>
       <c r="M4" t="n">
-        <v>0.7784</v>
+        <v>0.7712</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.7762</v>
+        <v>0.7658</v>
       </c>
     </row>
     <row r="5">
@@ -892,31 +892,31 @@
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0309</v>
+        <v>0.0289</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0394</v>
+        <v>0.0358</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.0346</v>
+        <v>0.032</v>
       </c>
       <c r="I5" t="n">
-        <v>0.128</v>
+        <v>0.1253</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1232</v>
+        <v>0.1084</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>0.1256</v>
+        <v>0.1163</v>
       </c>
       <c r="L5" t="n">
-        <v>0.7147</v>
+        <v>0.701</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7344000000000001</v>
+        <v>0.708</v>
       </c>
       <c r="N5" s="9" t="n">
-        <v>0.7244</v>
+        <v>0.7045</v>
       </c>
     </row>
     <row r="6">
@@ -936,37 +936,37 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>0.06950000000000001</v>
+        <v>0.7002</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0234</v>
+        <v>0.3367</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.035</v>
+        <v>0.4547</v>
       </c>
       <c r="I6" t="n">
-        <v>0.413</v>
+        <v>0.6833</v>
       </c>
       <c r="J6" t="n">
-        <v>0.2088</v>
+        <v>0.5076000000000001</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>0.2774</v>
+        <v>0.5825</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8733</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>0.7701</v>
+        <v>0.8743</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>0.8185</v>
+        <v>0.9046</v>
       </c>
     </row>
     <row r="7">
@@ -986,37 +986,37 @@
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0067</v>
+        <v>0.1629</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0025</v>
+        <v>0.2036</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.0036</v>
+        <v>0.181</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1788</v>
+        <v>0.3821</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1152</v>
+        <v>0.4271</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>0.1401</v>
+        <v>0.4034</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7013</v>
+        <v>0.7858000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>0.6549</v>
+        <v>0.797</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>0.6773</v>
+        <v>0.7914</v>
       </c>
     </row>
     <row r="8">
@@ -1036,37 +1036,37 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0063</v>
+        <v>0.32</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0028</v>
+        <v>0.2042</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.0039</v>
+        <v>0.2493</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1184</v>
+        <v>0.3805</v>
       </c>
       <c r="J8" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.2849</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.3258</v>
       </c>
       <c r="L8" t="n">
-        <v>0.75</v>
+        <v>0.8473000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>0.728</v>
+        <v>0.8307</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>0.7388</v>
+        <v>0.8389</v>
       </c>
     </row>
     <row r="9">
@@ -1086,37 +1086,37 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E9" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0731</v>
+        <v>0.0998</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.0708</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2218</v>
+        <v>0.2359</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2313</v>
+        <v>0.3221</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>0.2264</v>
+        <v>0.2723</v>
       </c>
       <c r="L9" t="n">
-        <v>0.7534</v>
+        <v>0.7437</v>
       </c>
       <c r="M9" t="n">
-        <v>0.7438</v>
+        <v>0.7784</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>0.7486</v>
+        <v>0.7606000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -1142,31 +1142,31 @@
         <v>4</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>0.3195</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>0.0799</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0</v>
+        <v>0.1278</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0958</v>
+        <v>0.501</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0689</v>
+        <v>0.2402</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>0.08019999999999999</v>
+        <v>0.3247</v>
       </c>
       <c r="L10" t="n">
-        <v>0.8167</v>
+        <v>0.876</v>
       </c>
       <c r="M10" t="n">
-        <v>0.7313</v>
+        <v>0.7571</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>0.7716</v>
+        <v>0.8122</v>
       </c>
     </row>
     <row r="11">
@@ -1186,37 +1186,37 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>0.3076</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>0.2769</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0</v>
+        <v>0.2915</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1047</v>
+        <v>0.4605</v>
       </c>
       <c r="J11" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.418</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>0.0987</v>
+        <v>0.4382</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6675</v>
+        <v>0.8397</v>
       </c>
       <c r="M11" t="n">
-        <v>0.6531</v>
+        <v>0.8157</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>0.6602</v>
+        <v>0.8275</v>
       </c>
     </row>
     <row r="12">
@@ -1251,22 +1251,22 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0951</v>
+        <v>0.2623</v>
       </c>
       <c r="J12" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.2814</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>0.0929</v>
+        <v>0.2715</v>
       </c>
       <c r="L12" t="n">
-        <v>0.7433</v>
+        <v>0.7748</v>
       </c>
       <c r="M12" t="n">
-        <v>0.7583</v>
+        <v>0.7785</v>
       </c>
       <c r="N12" s="9" t="n">
-        <v>0.7507</v>
+        <v>0.7766999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1292,31 +1292,31 @@
         <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>0.0582</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>0.0785</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0</v>
+        <v>0.0669</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1473</v>
+        <v>0.3219</v>
       </c>
       <c r="J13" t="n">
-        <v>0.1596</v>
+        <v>0.3694</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>0.1532</v>
+        <v>0.344</v>
       </c>
       <c r="L13" t="n">
-        <v>0.7102000000000001</v>
+        <v>0.7507</v>
       </c>
       <c r="M13" t="n">
-        <v>0.7187</v>
+        <v>0.759</v>
       </c>
       <c r="N13" s="9" t="n">
-        <v>0.7144</v>
+        <v>0.7548</v>
       </c>
     </row>
     <row r="14">
@@ -1342,31 +1342,31 @@
         <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0252</v>
+        <v>0.0503</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0551</v>
+        <v>0.074</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.0345</v>
+        <v>0.0599</v>
       </c>
       <c r="I14" t="n">
-        <v>0.1791</v>
+        <v>0.1732</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1506</v>
+        <v>0.1572</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>0.1636</v>
+        <v>0.1648</v>
       </c>
       <c r="L14" t="n">
-        <v>0.7376</v>
+        <v>0.7528</v>
       </c>
       <c r="M14" t="n">
-        <v>0.7451</v>
+        <v>0.7652</v>
       </c>
       <c r="N14" s="9" t="n">
-        <v>0.7413</v>
+        <v>0.7589</v>
       </c>
     </row>
     <row r="15">
@@ -1386,37 +1386,37 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0036</v>
+        <v>0.0398</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0009</v>
+        <v>0.0498</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.0014</v>
+        <v>0.0442</v>
       </c>
       <c r="I15" t="n">
-        <v>0.166</v>
+        <v>0.1981</v>
       </c>
       <c r="J15" t="n">
-        <v>0.0756</v>
+        <v>0.1993</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>0.1039</v>
+        <v>0.1987</v>
       </c>
       <c r="L15" t="n">
-        <v>0.7024</v>
+        <v>0.7731</v>
       </c>
       <c r="M15" t="n">
-        <v>0.6633</v>
+        <v>0.7879</v>
       </c>
       <c r="N15" s="9" t="n">
-        <v>0.6823</v>
+        <v>0.7804</v>
       </c>
     </row>
     <row r="16">
@@ -1436,37 +1436,37 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E16" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0062</v>
+        <v>0.0504</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0031</v>
+        <v>0.1151</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.0041</v>
+        <v>0.0701</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1763</v>
+        <v>0.2925</v>
       </c>
       <c r="J16" t="n">
-        <v>0.0921</v>
+        <v>0.3554</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>0.121</v>
+        <v>0.3209</v>
       </c>
       <c r="L16" t="n">
-        <v>0.7389</v>
+        <v>0.7659</v>
       </c>
       <c r="M16" t="n">
-        <v>0.6886</v>
+        <v>0.7916</v>
       </c>
       <c r="N16" s="9" t="n">
-        <v>0.7129</v>
+        <v>0.7785</v>
       </c>
     </row>
     <row r="17">
@@ -1486,37 +1486,37 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0502</v>
+        <v>0.0815</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0436</v>
+        <v>0.0977</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.0467</v>
+        <v>0.08890000000000001</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1932</v>
+        <v>0.2984</v>
       </c>
       <c r="J17" t="n">
-        <v>0.174</v>
+        <v>0.3506</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>0.1831</v>
+        <v>0.3224</v>
       </c>
       <c r="L17" t="n">
-        <v>0.7507</v>
+        <v>0.7343</v>
       </c>
       <c r="M17" t="n">
-        <v>0.7547</v>
+        <v>0.7443</v>
       </c>
       <c r="N17" s="9" t="n">
-        <v>0.7527</v>
+        <v>0.7393</v>
       </c>
     </row>
     <row r="18">
@@ -1536,37 +1536,37 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0111</v>
+        <v>0.3966</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0056</v>
+        <v>0.3502</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.0074</v>
+        <v>0.3719</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2155</v>
+        <v>0.5778</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1328</v>
+        <v>0.48</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>0.1643</v>
+        <v>0.5244</v>
       </c>
       <c r="L18" t="n">
-        <v>0.8066</v>
+        <v>0.8567</v>
       </c>
       <c r="M18" t="n">
-        <v>0.7441</v>
+        <v>0.8556</v>
       </c>
       <c r="N18" s="9" t="n">
-        <v>0.7741</v>
+        <v>0.8562</v>
       </c>
     </row>
     <row r="19">
@@ -1592,31 +1592,31 @@
         <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0426</v>
+        <v>0.0265</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0338</v>
+        <v>0.0124</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.0377</v>
+        <v>0.0169</v>
       </c>
       <c r="I19" t="n">
-        <v>0.2293</v>
+        <v>0.2049</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2011</v>
+        <v>0.1785</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>0.2143</v>
+        <v>0.1908</v>
       </c>
       <c r="L19" t="n">
-        <v>0.7527</v>
+        <v>0.7474</v>
       </c>
       <c r="M19" t="n">
-        <v>0.7597</v>
+        <v>0.7554999999999999</v>
       </c>
       <c r="N19" s="9" t="n">
-        <v>0.7562</v>
+        <v>0.7514</v>
       </c>
     </row>
     <row r="20">
@@ -1642,31 +1642,31 @@
         <v>4</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0725</v>
+        <v>0.0755</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0363</v>
+        <v>0.0549</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.0484</v>
+        <v>0.0636</v>
       </c>
       <c r="I20" t="n">
         <v>0.1058</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0898</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.1005</v>
       </c>
       <c r="L20" t="n">
-        <v>0.7721</v>
+        <v>0.7825</v>
       </c>
       <c r="M20" t="n">
-        <v>0.7544999999999999</v>
+        <v>0.7511</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>0.7632</v>
+        <v>0.7665</v>
       </c>
     </row>
     <row r="21">
@@ -1686,37 +1686,37 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0519</v>
+        <v>0.0701</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0693</v>
+        <v>0.0929</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.0593</v>
+        <v>0.0799</v>
       </c>
       <c r="I21" t="n">
-        <v>0.2198</v>
+        <v>0.2284</v>
       </c>
       <c r="J21" t="n">
-        <v>0.2389</v>
+        <v>0.2565</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>0.229</v>
+        <v>0.2416</v>
       </c>
       <c r="L21" t="n">
-        <v>0.7368</v>
+        <v>0.7257</v>
       </c>
       <c r="M21" t="n">
-        <v>0.7558</v>
+        <v>0.7469</v>
       </c>
       <c r="N21" s="9" t="n">
-        <v>0.7462</v>
+        <v>0.7362</v>
       </c>
     </row>
     <row r="22">
@@ -1786,37 +1786,37 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0075</v>
+        <v>0.1468</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0022</v>
+        <v>0.1608</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.0034</v>
+        <v>0.1535</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1438</v>
+        <v>0.2756</v>
       </c>
       <c r="J23" t="n">
-        <v>0.07969999999999999</v>
+        <v>0.2483</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>0.1026</v>
+        <v>0.2612</v>
       </c>
       <c r="L23" t="n">
-        <v>0.7046</v>
+        <v>0.7975</v>
       </c>
       <c r="M23" t="n">
-        <v>0.6868</v>
+        <v>0.799</v>
       </c>
       <c r="N23" s="9" t="n">
-        <v>0.6955</v>
+        <v>0.7982</v>
       </c>
     </row>
     <row r="24">
@@ -1854,19 +1854,19 @@
         <v>0.2711</v>
       </c>
       <c r="J24" t="n">
-        <v>0.1413</v>
+        <v>0.1397</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>0.1858</v>
+        <v>0.1844</v>
       </c>
       <c r="L24" t="n">
         <v>0.8347</v>
       </c>
       <c r="M24" t="n">
-        <v>0.7781</v>
+        <v>0.7728</v>
       </c>
       <c r="N24" s="9" t="n">
-        <v>0.8054</v>
+        <v>0.8026</v>
       </c>
     </row>
     <row r="25">
@@ -1886,37 +1886,37 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0606</v>
+        <v>0.0524</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0433</v>
+        <v>0.07969999999999999</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.0505</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="I25" t="n">
-        <v>0.2453</v>
+        <v>0.1643</v>
       </c>
       <c r="J25" t="n">
-        <v>0.1628</v>
+        <v>0.193</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>0.1957</v>
+        <v>0.1775</v>
       </c>
       <c r="L25" t="n">
-        <v>0.7747000000000001</v>
+        <v>0.7073</v>
       </c>
       <c r="M25" t="n">
-        <v>0.7358</v>
+        <v>0.7412</v>
       </c>
       <c r="N25" s="9" t="n">
-        <v>0.7547</v>
+        <v>0.7239</v>
       </c>
     </row>
     <row r="26">
@@ -1936,37 +1936,37 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>0.0149</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>0.0133</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0</v>
+        <v>0.0141</v>
       </c>
       <c r="I26" t="n">
-        <v>0.0333</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0221</v>
+        <v>0.0733</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>0.0266</v>
+        <v>0.0779</v>
       </c>
       <c r="L26" t="n">
-        <v>0.6556</v>
+        <v>0.723</v>
       </c>
       <c r="M26" t="n">
-        <v>0.6469</v>
+        <v>0.7331</v>
       </c>
       <c r="N26" s="9" t="n">
-        <v>0.6512</v>
+        <v>0.728</v>
       </c>
     </row>
     <row r="27">
@@ -2001,22 +2001,22 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>0.0607</v>
+        <v>0.0717</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0562</v>
+        <v>0.0498</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>0.0583</v>
+        <v>0.0588</v>
       </c>
       <c r="L27" t="n">
-        <v>0.7257</v>
+        <v>0.7019</v>
       </c>
       <c r="M27" t="n">
-        <v>0.6749000000000001</v>
+        <v>0.6567</v>
       </c>
       <c r="N27" s="9" t="n">
-        <v>0.6994</v>
+        <v>0.6785</v>
       </c>
     </row>
     <row r="28">
@@ -2036,37 +2036,37 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E28" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>0.0919</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>0.062</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0</v>
+        <v>0.0741</v>
       </c>
       <c r="I28" t="n">
-        <v>0.08459999999999999</v>
+        <v>0.1112</v>
       </c>
       <c r="J28" t="n">
-        <v>0.09429999999999999</v>
+        <v>0.1094</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>0.0892</v>
+        <v>0.1103</v>
       </c>
       <c r="L28" t="n">
-        <v>0.7367</v>
+        <v>0.7783</v>
       </c>
       <c r="M28" t="n">
-        <v>0.7289</v>
+        <v>0.7661</v>
       </c>
       <c r="N28" s="9" t="n">
-        <v>0.7327</v>
+        <v>0.7721</v>
       </c>
     </row>
     <row r="29">
@@ -2092,31 +2092,31 @@
         <v>4</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0363</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0689</v>
+        <v>0.0578</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.0475</v>
+        <v>0.0606</v>
       </c>
       <c r="I29" t="n">
-        <v>0.1386</v>
+        <v>0.1687</v>
       </c>
       <c r="J29" t="n">
-        <v>0.1108</v>
+        <v>0.1484</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>0.1231</v>
+        <v>0.1579</v>
       </c>
       <c r="L29" t="n">
-        <v>0.703</v>
+        <v>0.7088</v>
       </c>
       <c r="M29" t="n">
-        <v>0.6989</v>
+        <v>0.7032</v>
       </c>
       <c r="N29" s="9" t="n">
-        <v>0.701</v>
+        <v>0.706</v>
       </c>
     </row>
     <row r="30">
@@ -2142,31 +2142,31 @@
         <v>4</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>0.0877</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>0.0457</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0</v>
+        <v>0.0601</v>
       </c>
       <c r="I30" t="n">
-        <v>0.1393</v>
+        <v>0.3716</v>
       </c>
       <c r="J30" t="n">
-        <v>0.1231</v>
+        <v>0.2395</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>0.1307</v>
+        <v>0.2913</v>
       </c>
       <c r="L30" t="n">
-        <v>0.7143</v>
+        <v>0.7399</v>
       </c>
       <c r="M30" t="n">
-        <v>0.7454</v>
+        <v>0.7429</v>
       </c>
       <c r="N30" s="9" t="n">
-        <v>0.7295</v>
+        <v>0.7413999999999999</v>
       </c>
     </row>
     <row r="31">
@@ -2186,37 +2186,37 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>0.6988</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>0.3987</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0</v>
+        <v>0.5077</v>
       </c>
       <c r="I31" t="n">
-        <v>0.1393</v>
+        <v>0.9414</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0912</v>
+        <v>0.5919</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>0.1102</v>
+        <v>0.7268</v>
       </c>
       <c r="L31" t="n">
-        <v>0.7582</v>
+        <v>0.9585</v>
       </c>
       <c r="M31" t="n">
-        <v>0.7329</v>
+        <v>0.879</v>
       </c>
       <c r="N31" s="9" t="n">
-        <v>0.7453</v>
+        <v>0.917</v>
       </c>
     </row>
     <row r="32">
@@ -2242,31 +2242,31 @@
         <v>4</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>0.048</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>0.0349</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0</v>
+        <v>0.0404</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1001</v>
+        <v>0.1531</v>
       </c>
       <c r="J32" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.135</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>0.0834</v>
+        <v>0.1435</v>
       </c>
       <c r="L32" t="n">
-        <v>0.6977</v>
+        <v>0.745</v>
       </c>
       <c r="M32" t="n">
-        <v>0.6791</v>
+        <v>0.7249</v>
       </c>
       <c r="N32" s="9" t="n">
-        <v>0.6883</v>
+        <v>0.7348</v>
       </c>
     </row>
     <row r="33">
@@ -2286,37 +2286,37 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>0.0523</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>0.06510000000000001</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0</v>
+        <v>0.058</v>
       </c>
       <c r="I33" t="n">
-        <v>0.1044</v>
+        <v>0.1766</v>
       </c>
       <c r="J33" t="n">
-        <v>0.1041</v>
+        <v>0.218</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>0.1043</v>
+        <v>0.1951</v>
       </c>
       <c r="L33" t="n">
-        <v>0.6499</v>
+        <v>0.7247</v>
       </c>
       <c r="M33" t="n">
-        <v>0.6292</v>
+        <v>0.7417</v>
       </c>
       <c r="N33" s="9" t="n">
-        <v>0.6394</v>
+        <v>0.7331</v>
       </c>
     </row>
     <row r="34">
@@ -2336,37 +2336,37 @@
         </is>
       </c>
       <c r="D34" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E34" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>0.0706</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>0.1017</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0</v>
+        <v>0.0834</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1019</v>
+        <v>0.1258</v>
       </c>
       <c r="J34" t="n">
-        <v>0.097</v>
+        <v>0.1326</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>0.0994</v>
+        <v>0.1291</v>
       </c>
       <c r="L34" t="n">
-        <v>0.6902</v>
+        <v>0.7157</v>
       </c>
       <c r="M34" t="n">
-        <v>0.7040999999999999</v>
+        <v>0.7274</v>
       </c>
       <c r="N34" s="9" t="n">
-        <v>0.6971000000000001</v>
+        <v>0.7215</v>
       </c>
     </row>
     <row r="35">
@@ -2392,31 +2392,31 @@
         <v>4</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>0.0425</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>0.0611</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0</v>
+        <v>0.0501</v>
       </c>
       <c r="I35" t="n">
-        <v>0.083</v>
+        <v>0.1218</v>
       </c>
       <c r="J35" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.1773</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>0.09039999999999999</v>
+        <v>0.1444</v>
       </c>
       <c r="L35" t="n">
-        <v>0.6821</v>
+        <v>0.7229</v>
       </c>
       <c r="M35" t="n">
-        <v>0.7123</v>
+        <v>0.7662</v>
       </c>
       <c r="N35" s="9" t="n">
-        <v>0.6969</v>
+        <v>0.7439</v>
       </c>
     </row>
     <row r="36">
@@ -2436,37 +2436,37 @@
         </is>
       </c>
       <c r="D36" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E36" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>0.0688</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>0.0688</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0</v>
+        <v>0.0688</v>
       </c>
       <c r="I36" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.2891</v>
       </c>
       <c r="J36" t="n">
-        <v>0.0793</v>
+        <v>0.3037</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.2962</v>
       </c>
       <c r="L36" t="n">
-        <v>0.6909</v>
+        <v>0.7886</v>
       </c>
       <c r="M36" t="n">
-        <v>0.6798999999999999</v>
+        <v>0.8022</v>
       </c>
       <c r="N36" s="9" t="n">
-        <v>0.6853</v>
+        <v>0.7954</v>
       </c>
     </row>
     <row r="37">
@@ -2486,37 +2486,37 @@
         </is>
       </c>
       <c r="D37" s="8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E37" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F37" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0281</v>
       </c>
       <c r="G37" t="n">
-        <v>0.0187</v>
+        <v>0.044</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.0119</v>
+        <v>0.0343</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0795</v>
+        <v>0.133</v>
       </c>
       <c r="J37" t="n">
-        <v>0.08450000000000001</v>
+        <v>0.1448</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>0.0819</v>
+        <v>0.1387</v>
       </c>
       <c r="L37" t="n">
-        <v>0.6675</v>
+        <v>0.7126</v>
       </c>
       <c r="M37" t="n">
-        <v>0.678</v>
+        <v>0.7339</v>
       </c>
       <c r="N37" s="9" t="n">
-        <v>0.6727</v>
+        <v>0.7231</v>
       </c>
     </row>
     <row r="38">
@@ -2542,31 +2542,31 @@
         <v>4</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>0.5503</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>0.1643</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0</v>
+        <v>0.253</v>
       </c>
       <c r="I38" t="n">
-        <v>0.0743</v>
+        <v>0.4385</v>
       </c>
       <c r="J38" t="n">
-        <v>0.064</v>
+        <v>0.2005</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>0.0687</v>
+        <v>0.2752</v>
       </c>
       <c r="L38" t="n">
-        <v>0.7663</v>
+        <v>0.8696</v>
       </c>
       <c r="M38" t="n">
-        <v>0.7314000000000001</v>
+        <v>0.7859</v>
       </c>
       <c r="N38" s="9" t="n">
-        <v>0.7485000000000001</v>
+        <v>0.8256</v>
       </c>
     </row>
     <row r="39">
@@ -2592,31 +2592,31 @@
         <v>4</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>0.1057</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0</v>
+        <v>0.09760000000000001</v>
       </c>
       <c r="I39" t="n">
-        <v>0.1223</v>
+        <v>0.2761</v>
       </c>
       <c r="J39" t="n">
-        <v>0.1272</v>
+        <v>0.2879</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>0.1247</v>
+        <v>0.2819</v>
       </c>
       <c r="L39" t="n">
-        <v>0.7206</v>
+        <v>0.7802</v>
       </c>
       <c r="M39" t="n">
-        <v>0.7366</v>
+        <v>0.7829</v>
       </c>
       <c r="N39" s="9" t="n">
-        <v>0.7285</v>
+        <v>0.7815</v>
       </c>
     </row>
     <row r="40">
@@ -2642,31 +2642,31 @@
         <v>4</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>0.1068</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>0.0801</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0</v>
+        <v>0.0916</v>
       </c>
       <c r="I40" t="n">
-        <v>0.0896</v>
+        <v>0.2004</v>
       </c>
       <c r="J40" t="n">
-        <v>0.07439999999999999</v>
+        <v>0.1441</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>0.0813</v>
+        <v>0.1677</v>
       </c>
       <c r="L40" t="n">
-        <v>0.7382</v>
+        <v>0.7963</v>
       </c>
       <c r="M40" t="n">
-        <v>0.7213000000000001</v>
+        <v>0.7781</v>
       </c>
       <c r="N40" s="9" t="n">
-        <v>0.7296</v>
+        <v>0.7871</v>
       </c>
     </row>
     <row r="41">
@@ -2692,31 +2692,31 @@
         <v>4</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>0.0261</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>0.0344</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0</v>
+        <v>0.0297</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0969</v>
+        <v>0.1225</v>
       </c>
       <c r="J41" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.1303</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>0.0871</v>
+        <v>0.1263</v>
       </c>
       <c r="L41" t="n">
-        <v>0.6991000000000001</v>
+        <v>0.7313</v>
       </c>
       <c r="M41" t="n">
-        <v>0.6894</v>
+        <v>0.7346</v>
       </c>
       <c r="N41" s="9" t="n">
-        <v>0.6942</v>
+        <v>0.7329</v>
       </c>
     </row>
     <row r="42">
@@ -2736,37 +2736,37 @@
         </is>
       </c>
       <c r="D42" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F42" t="n">
-        <v>0.2825</v>
+        <v>0.4127</v>
       </c>
       <c r="G42" t="n">
-        <v>0.1017</v>
+        <v>0.2463</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.1496</v>
+        <v>0.3085</v>
       </c>
       <c r="I42" t="n">
-        <v>0.4976</v>
+        <v>0.795</v>
       </c>
       <c r="J42" t="n">
-        <v>0.2337</v>
+        <v>0.4513</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>0.318</v>
+        <v>0.5758</v>
       </c>
       <c r="L42" t="n">
-        <v>0.832</v>
+        <v>0.8888</v>
       </c>
       <c r="M42" t="n">
-        <v>0.7509</v>
+        <v>0.8428</v>
       </c>
       <c r="N42" s="9" t="n">
-        <v>0.7894</v>
+        <v>0.8652</v>
       </c>
     </row>
     <row r="43">
@@ -2786,37 +2786,37 @@
         </is>
       </c>
       <c r="D43" s="8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E43" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>0.0282</v>
       </c>
       <c r="G43" t="n">
-        <v>0</v>
+        <v>0.08450000000000001</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0</v>
+        <v>0.0422</v>
       </c>
       <c r="I43" t="n">
-        <v>0.0453</v>
+        <v>0.141</v>
       </c>
       <c r="J43" t="n">
-        <v>0.0409</v>
+        <v>0.1756</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>0.043</v>
+        <v>0.1564</v>
       </c>
       <c r="L43" t="n">
-        <v>0.6491</v>
+        <v>0.729</v>
       </c>
       <c r="M43" t="n">
-        <v>0.6348</v>
+        <v>0.7758</v>
       </c>
       <c r="N43" s="9" t="n">
-        <v>0.6419</v>
+        <v>0.7517</v>
       </c>
     </row>
     <row r="44">
@@ -2836,37 +2836,37 @@
         </is>
       </c>
       <c r="D44" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F44" t="n">
-        <v>0.0029</v>
+        <v>0.0305</v>
       </c>
       <c r="G44" t="n">
-        <v>0.0013</v>
+        <v>0.0178</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.0018</v>
+        <v>0.0225</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0794</v>
+        <v>0.1373</v>
       </c>
       <c r="J44" t="n">
-        <v>0.0591</v>
+        <v>0.1075</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>0.0678</v>
+        <v>0.1206</v>
       </c>
       <c r="L44" t="n">
-        <v>0.7149</v>
+        <v>0.7359</v>
       </c>
       <c r="M44" t="n">
-        <v>0.6883</v>
+        <v>0.7183</v>
       </c>
       <c r="N44" s="9" t="n">
-        <v>0.7014</v>
+        <v>0.727</v>
       </c>
     </row>
     <row r="45">
@@ -2901,22 +2901,22 @@
         <v>0.0325</v>
       </c>
       <c r="I45" t="n">
-        <v>0.3729</v>
+        <v>0.376</v>
       </c>
       <c r="J45" t="n">
-        <v>0.1551</v>
+        <v>0.1696</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>0.2191</v>
+        <v>0.2337</v>
       </c>
       <c r="L45" t="n">
-        <v>0.746</v>
+        <v>0.7485000000000001</v>
       </c>
       <c r="M45" t="n">
-        <v>0.6794</v>
+        <v>0.699</v>
       </c>
       <c r="N45" s="9" t="n">
-        <v>0.7112000000000001</v>
+        <v>0.7229</v>
       </c>
     </row>
     <row r="46">
@@ -2942,31 +2942,31 @@
         <v>4</v>
       </c>
       <c r="F46" t="n">
-        <v>0.2628</v>
+        <v>0.1928</v>
       </c>
       <c r="G46" t="n">
-        <v>0.1886</v>
+        <v>0.1691</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.2196</v>
+        <v>0.1802</v>
       </c>
       <c r="I46" t="n">
-        <v>0.2289</v>
+        <v>0.2133</v>
       </c>
       <c r="J46" t="n">
-        <v>0.1692</v>
+        <v>0.16</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>0.1946</v>
+        <v>0.1829</v>
       </c>
       <c r="L46" t="n">
-        <v>0.8077</v>
+        <v>0.7892</v>
       </c>
       <c r="M46" t="n">
-        <v>0.79</v>
+        <v>0.7897999999999999</v>
       </c>
       <c r="N46" s="9" t="n">
-        <v>0.7987</v>
+        <v>0.7895</v>
       </c>
     </row>
     <row r="47">
@@ -2986,37 +2986,37 @@
         </is>
       </c>
       <c r="D47" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E47" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0003</v>
+        <v>0.0374</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0001</v>
+        <v>0.0474</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.0002</v>
+        <v>0.0418</v>
       </c>
       <c r="I47" t="n">
-        <v>0.0638</v>
+        <v>0.1551</v>
       </c>
       <c r="J47" t="n">
-        <v>0.0485</v>
+        <v>0.1601</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>0.0551</v>
+        <v>0.1575</v>
       </c>
       <c r="L47" t="n">
-        <v>0.6561</v>
+        <v>0.7328</v>
       </c>
       <c r="M47" t="n">
-        <v>0.6462</v>
+        <v>0.74</v>
       </c>
       <c r="N47" s="9" t="n">
-        <v>0.6511</v>
+        <v>0.7364000000000001</v>
       </c>
     </row>
     <row r="48">
@@ -3051,22 +3051,22 @@
         <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>0.107</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="J48" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.0677</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>0.0926</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="L48" t="n">
-        <v>0.7413</v>
+        <v>0.7569</v>
       </c>
       <c r="M48" t="n">
-        <v>0.7287</v>
+        <v>0.7359</v>
       </c>
       <c r="N48" s="9" t="n">
-        <v>0.735</v>
+        <v>0.7463</v>
       </c>
     </row>
     <row r="49">
@@ -3086,37 +3086,37 @@
         </is>
       </c>
       <c r="D49" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0281</v>
+        <v>0.059</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0151</v>
+        <v>0.0578</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.0196</v>
+        <v>0.0584</v>
       </c>
       <c r="I49" t="n">
-        <v>0.1785</v>
+        <v>0.1932</v>
       </c>
       <c r="J49" t="n">
-        <v>0.1156</v>
+        <v>0.1519</v>
       </c>
       <c r="K49" s="9" t="n">
-        <v>0.1403</v>
+        <v>0.1701</v>
       </c>
       <c r="L49" t="n">
-        <v>0.6881</v>
+        <v>0.7023</v>
       </c>
       <c r="M49" t="n">
-        <v>0.6691</v>
+        <v>0.7019</v>
       </c>
       <c r="N49" s="9" t="n">
-        <v>0.6785</v>
+        <v>0.7020999999999999</v>
       </c>
     </row>
     <row r="50">
@@ -3136,37 +3136,37 @@
         </is>
       </c>
       <c r="D50" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F50" t="n">
-        <v>0.0267</v>
+        <v>0.1692</v>
       </c>
       <c r="G50" t="n">
-        <v>0.0067</v>
+        <v>0.0493</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.0107</v>
+        <v>0.07630000000000001</v>
       </c>
       <c r="I50" t="n">
-        <v>0.09080000000000001</v>
+        <v>0.1279</v>
       </c>
       <c r="J50" t="n">
-        <v>0.0688</v>
+        <v>0.1116</v>
       </c>
       <c r="K50" s="9" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.1192</v>
       </c>
       <c r="L50" t="n">
-        <v>0.6777</v>
+        <v>0.7183</v>
       </c>
       <c r="M50" t="n">
-        <v>0.669</v>
+        <v>0.7221</v>
       </c>
       <c r="N50" s="9" t="n">
-        <v>0.6734</v>
+        <v>0.7202</v>
       </c>
     </row>
     <row r="51">
@@ -3186,37 +3186,37 @@
         </is>
       </c>
       <c r="D51" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E51" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F51" t="n">
-        <v>0.0003</v>
+        <v>0.0392</v>
       </c>
       <c r="G51" t="n">
-        <v>0.0001</v>
+        <v>0.033</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.0002</v>
+        <v>0.0358</v>
       </c>
       <c r="I51" t="n">
-        <v>0.1098</v>
+        <v>0.2527</v>
       </c>
       <c r="J51" t="n">
-        <v>0.0624</v>
+        <v>0.1769</v>
       </c>
       <c r="K51" s="9" t="n">
-        <v>0.0796</v>
+        <v>0.2081</v>
       </c>
       <c r="L51" t="n">
-        <v>0.7217</v>
+        <v>0.7492</v>
       </c>
       <c r="M51" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.7423</v>
       </c>
       <c r="N51" s="9" t="n">
-        <v>0.707</v>
+        <v>0.7457</v>
       </c>
     </row>
     <row r="52">
@@ -3236,37 +3236,37 @@
         </is>
       </c>
       <c r="D52" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E52" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F52" t="n">
-        <v>0.0062</v>
+        <v>0.06510000000000001</v>
       </c>
       <c r="G52" t="n">
-        <v>0.0046</v>
+        <v>0.0578</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.0053</v>
+        <v>0.0612</v>
       </c>
       <c r="I52" t="n">
-        <v>0.1053</v>
+        <v>0.1242</v>
       </c>
       <c r="J52" t="n">
-        <v>0.0639</v>
+        <v>0.1056</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>0.0795</v>
+        <v>0.1142</v>
       </c>
       <c r="L52" t="n">
-        <v>0.7282999999999999</v>
+        <v>0.7838000000000001</v>
       </c>
       <c r="M52" t="n">
-        <v>0.7138</v>
+        <v>0.7938</v>
       </c>
       <c r="N52" s="9" t="n">
-        <v>0.721</v>
+        <v>0.7887999999999999</v>
       </c>
     </row>
     <row r="53">
@@ -3301,22 +3301,22 @@
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>0.1324</v>
+        <v>0.1481</v>
       </c>
       <c r="J53" t="n">
-        <v>0.0974</v>
+        <v>0.1133</v>
       </c>
       <c r="K53" s="9" t="n">
-        <v>0.1122</v>
+        <v>0.1284</v>
       </c>
       <c r="L53" t="n">
-        <v>0.6609</v>
+        <v>0.6694</v>
       </c>
       <c r="M53" t="n">
-        <v>0.6489</v>
+        <v>0.6483</v>
       </c>
       <c r="N53" s="9" t="n">
-        <v>0.6549</v>
+        <v>0.6587</v>
       </c>
     </row>
     <row r="54">
@@ -3336,37 +3336,37 @@
         </is>
       </c>
       <c r="D54" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E54" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F54" t="n">
-        <v>0.1451</v>
+        <v>0.1972</v>
       </c>
       <c r="G54" t="n">
-        <v>0.0544</v>
+        <v>0.1479</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.0791</v>
+        <v>0.169</v>
       </c>
       <c r="I54" t="n">
-        <v>0.3667</v>
+        <v>0.5927</v>
       </c>
       <c r="J54" t="n">
-        <v>0.2184</v>
+        <v>0.3843</v>
       </c>
       <c r="K54" s="9" t="n">
-        <v>0.2737</v>
+        <v>0.4663</v>
       </c>
       <c r="L54" t="n">
-        <v>0.8074</v>
+        <v>0.8397</v>
       </c>
       <c r="M54" t="n">
-        <v>0.7614</v>
+        <v>0.8139</v>
       </c>
       <c r="N54" s="9" t="n">
-        <v>0.7837</v>
+        <v>0.8266</v>
       </c>
     </row>
     <row r="55">
@@ -3386,37 +3386,37 @@
         </is>
       </c>
       <c r="D55" s="8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E55" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F55" t="n">
-        <v>0</v>
+        <v>0.0172</v>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>0.0239</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="I55" t="n">
-        <v>0.0861</v>
+        <v>0.2025</v>
       </c>
       <c r="J55" t="n">
-        <v>0.0452</v>
+        <v>0.2027</v>
       </c>
       <c r="K55" s="9" t="n">
-        <v>0.0593</v>
+        <v>0.2026</v>
       </c>
       <c r="L55" t="n">
-        <v>0.7109</v>
+        <v>0.78</v>
       </c>
       <c r="M55" t="n">
-        <v>0.6461</v>
+        <v>0.7881</v>
       </c>
       <c r="N55" s="9" t="n">
-        <v>0.6768999999999999</v>
+        <v>0.784</v>
       </c>
     </row>
     <row r="56">
@@ -3436,37 +3436,37 @@
         </is>
       </c>
       <c r="D56" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E56" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F56" t="n">
-        <v>0.0014</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="G56" t="n">
-        <v>0.0004</v>
+        <v>0.1292</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.0007</v>
+        <v>0.0919</v>
       </c>
       <c r="I56" t="n">
-        <v>0.0518</v>
+        <v>0.1122</v>
       </c>
       <c r="J56" t="n">
-        <v>0.0364</v>
+        <v>0.112</v>
       </c>
       <c r="K56" s="9" t="n">
-        <v>0.0428</v>
+        <v>0.1121</v>
       </c>
       <c r="L56" t="n">
-        <v>0.6823</v>
+        <v>0.7661</v>
       </c>
       <c r="M56" t="n">
-        <v>0.6599</v>
+        <v>0.7761</v>
       </c>
       <c r="N56" s="9" t="n">
-        <v>0.6709000000000001</v>
+        <v>0.771</v>
       </c>
     </row>
     <row r="57">
@@ -3486,37 +3486,37 @@
         </is>
       </c>
       <c r="D57" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E57" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F57" t="n">
-        <v>0.0151</v>
+        <v>0.025</v>
       </c>
       <c r="G57" t="n">
-        <v>0.0097</v>
+        <v>0.0383</v>
       </c>
       <c r="H57" s="9" t="n">
-        <v>0.0118</v>
+        <v>0.0302</v>
       </c>
       <c r="I57" t="n">
-        <v>0.1138</v>
+        <v>0.142</v>
       </c>
       <c r="J57" t="n">
-        <v>0.1077</v>
+        <v>0.1453</v>
       </c>
       <c r="K57" s="9" t="n">
-        <v>0.1107</v>
+        <v>0.1437</v>
       </c>
       <c r="L57" t="n">
-        <v>0.7109</v>
+        <v>0.7029</v>
       </c>
       <c r="M57" t="n">
-        <v>0.6829</v>
+        <v>0.6981000000000001</v>
       </c>
       <c r="N57" s="9" t="n">
-        <v>0.6966</v>
+        <v>0.7005</v>
       </c>
     </row>
     <row r="58">
@@ -3536,37 +3536,37 @@
         </is>
       </c>
       <c r="D58" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E58" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F58" t="n">
-        <v>0.0144</v>
+        <v>0.2285</v>
       </c>
       <c r="G58" t="n">
-        <v>0.0211</v>
+        <v>0.2862</v>
       </c>
       <c r="H58" s="9" t="n">
-        <v>0.0171</v>
+        <v>0.2541</v>
       </c>
       <c r="I58" t="n">
-        <v>0.1222</v>
+        <v>0.3501</v>
       </c>
       <c r="J58" t="n">
-        <v>0.123</v>
+        <v>0.3648</v>
       </c>
       <c r="K58" s="9" t="n">
-        <v>0.1226</v>
+        <v>0.3573</v>
       </c>
       <c r="L58" t="n">
-        <v>0.7367</v>
+        <v>0.8091</v>
       </c>
       <c r="M58" t="n">
-        <v>0.7558</v>
+        <v>0.8493000000000001</v>
       </c>
       <c r="N58" s="9" t="n">
-        <v>0.7461</v>
+        <v>0.8287</v>
       </c>
     </row>
     <row r="59">
@@ -3586,37 +3586,37 @@
         </is>
       </c>
       <c r="D59" s="8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E59" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F59" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.1458</v>
       </c>
       <c r="G59" t="n">
-        <v>0.003</v>
+        <v>0.2124</v>
       </c>
       <c r="H59" s="9" t="n">
-        <v>0.0045</v>
+        <v>0.1729</v>
       </c>
       <c r="I59" t="n">
-        <v>0.119</v>
+        <v>0.2269</v>
       </c>
       <c r="J59" t="n">
-        <v>0.0907</v>
+        <v>0.3494</v>
       </c>
       <c r="K59" s="9" t="n">
-        <v>0.103</v>
+        <v>0.2751</v>
       </c>
       <c r="L59" t="n">
-        <v>0.695</v>
+        <v>0.7765</v>
       </c>
       <c r="M59" t="n">
-        <v>0.6729000000000001</v>
+        <v>0.839</v>
       </c>
       <c r="N59" s="9" t="n">
-        <v>0.6837</v>
+        <v>0.8066</v>
       </c>
     </row>
     <row r="60">
@@ -3636,37 +3636,37 @@
         </is>
       </c>
       <c r="D60" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E60" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F60" t="n">
-        <v>0.0214</v>
+        <v>0.0979</v>
       </c>
       <c r="G60" t="n">
-        <v>0.0256</v>
+        <v>0.1411</v>
       </c>
       <c r="H60" s="9" t="n">
-        <v>0.0233</v>
+        <v>0.1156</v>
       </c>
       <c r="I60" t="n">
-        <v>0.1177</v>
+        <v>0.1991</v>
       </c>
       <c r="J60" t="n">
-        <v>0.1017</v>
+        <v>0.2046</v>
       </c>
       <c r="K60" s="9" t="n">
-        <v>0.1091</v>
+        <v>0.2018</v>
       </c>
       <c r="L60" t="n">
-        <v>0.7498</v>
+        <v>0.7829</v>
       </c>
       <c r="M60" t="n">
-        <v>0.7582</v>
+        <v>0.8199</v>
       </c>
       <c r="N60" s="9" t="n">
-        <v>0.754</v>
+        <v>0.801</v>
       </c>
     </row>
     <row r="61">
@@ -3686,37 +3686,37 @@
         </is>
       </c>
       <c r="D61" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E61" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F61" t="n">
-        <v>0.0023</v>
+        <v>0.0244</v>
       </c>
       <c r="G61" t="n">
-        <v>0.0015</v>
+        <v>0.0206</v>
       </c>
       <c r="H61" s="9" t="n">
-        <v>0.0018</v>
+        <v>0.0223</v>
       </c>
       <c r="I61" t="n">
-        <v>0.1134</v>
+        <v>0.1637</v>
       </c>
       <c r="J61" t="n">
-        <v>0.0838</v>
+        <v>0.1488</v>
       </c>
       <c r="K61" s="9" t="n">
-        <v>0.0964</v>
+        <v>0.1559</v>
       </c>
       <c r="L61" t="n">
-        <v>0.6811</v>
+        <v>0.7058</v>
       </c>
       <c r="M61" t="n">
-        <v>0.6673</v>
+        <v>0.699</v>
       </c>
       <c r="N61" s="9" t="n">
-        <v>0.6742</v>
+        <v>0.7024</v>
       </c>
     </row>
     <row r="62">
@@ -3786,37 +3786,37 @@
         </is>
       </c>
       <c r="D63" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E63" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F63" t="n">
-        <v>0.0699</v>
+        <v>0.1283</v>
       </c>
       <c r="G63" t="n">
-        <v>0.0579</v>
+        <v>0.2034</v>
       </c>
       <c r="H63" s="9" t="n">
-        <v>0.0633</v>
+        <v>0.1573</v>
       </c>
       <c r="I63" t="n">
-        <v>0.1869</v>
+        <v>0.2119</v>
       </c>
       <c r="J63" t="n">
-        <v>0.1553</v>
+        <v>0.2774</v>
       </c>
       <c r="K63" s="9" t="n">
-        <v>0.1696</v>
+        <v>0.2403</v>
       </c>
       <c r="L63" t="n">
-        <v>0.7309</v>
+        <v>0.7675999999999999</v>
       </c>
       <c r="M63" t="n">
-        <v>0.7306</v>
+        <v>0.8101</v>
       </c>
       <c r="N63" s="9" t="n">
-        <v>0.7307</v>
+        <v>0.7883</v>
       </c>
     </row>
     <row r="64">
@@ -3842,31 +3842,31 @@
         <v>4</v>
       </c>
       <c r="F64" t="n">
-        <v>0.1169</v>
+        <v>0.094</v>
       </c>
       <c r="G64" t="n">
-        <v>0.0585</v>
+        <v>0.0508</v>
       </c>
       <c r="H64" s="9" t="n">
-        <v>0.078</v>
+        <v>0.066</v>
       </c>
       <c r="I64" t="n">
-        <v>0.246</v>
+        <v>0.2247</v>
       </c>
       <c r="J64" t="n">
-        <v>0.1447</v>
+        <v>0.1503</v>
       </c>
       <c r="K64" s="9" t="n">
-        <v>0.1822</v>
+        <v>0.1801</v>
       </c>
       <c r="L64" t="n">
-        <v>0.7873</v>
+        <v>0.7885</v>
       </c>
       <c r="M64" t="n">
-        <v>0.7832</v>
+        <v>0.79</v>
       </c>
       <c r="N64" s="9" t="n">
-        <v>0.7852</v>
+        <v>0.7892</v>
       </c>
     </row>
     <row r="65">
@@ -3892,31 +3892,31 @@
         <v>4</v>
       </c>
       <c r="F65" t="n">
-        <v>0.1269</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="G65" t="n">
-        <v>0.1198</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="H65" s="9" t="n">
-        <v>0.1232</v>
+        <v>0.0791</v>
       </c>
       <c r="I65" t="n">
-        <v>0.1884</v>
+        <v>0.1726</v>
       </c>
       <c r="J65" t="n">
-        <v>0.1484</v>
+        <v>0.1512</v>
       </c>
       <c r="K65" s="9" t="n">
-        <v>0.1661</v>
+        <v>0.1612</v>
       </c>
       <c r="L65" t="n">
-        <v>0.7342</v>
+        <v>0.7196</v>
       </c>
       <c r="M65" t="n">
-        <v>0.7137</v>
+        <v>0.7247</v>
       </c>
       <c r="N65" s="9" t="n">
-        <v>0.7238</v>
+        <v>0.7222</v>
       </c>
     </row>
     <row r="66">
@@ -3995,28 +3995,28 @@
         <v>0.0521</v>
       </c>
       <c r="G67" t="n">
-        <v>0.0435</v>
+        <v>0.0368</v>
       </c>
       <c r="H67" s="9" t="n">
-        <v>0.0474</v>
+        <v>0.0431</v>
       </c>
       <c r="I67" t="n">
         <v>0.1678</v>
       </c>
       <c r="J67" t="n">
-        <v>0.1291</v>
+        <v>0.1276</v>
       </c>
       <c r="K67" s="9" t="n">
-        <v>0.1459</v>
+        <v>0.1449</v>
       </c>
       <c r="L67" t="n">
         <v>0.7635999999999999</v>
       </c>
       <c r="M67" t="n">
-        <v>0.7313</v>
+        <v>0.7321</v>
       </c>
       <c r="N67" s="9" t="n">
-        <v>0.7471</v>
+        <v>0.7475000000000001</v>
       </c>
     </row>
     <row r="68">
@@ -4054,19 +4054,19 @@
         <v>0.0977</v>
       </c>
       <c r="J68" t="n">
-        <v>0.0774</v>
+        <v>0.0765</v>
       </c>
       <c r="K68" s="9" t="n">
-        <v>0.0864</v>
+        <v>0.0858</v>
       </c>
       <c r="L68" t="n">
-        <v>0.7219</v>
+        <v>0.7367</v>
       </c>
       <c r="M68" t="n">
-        <v>0.7007</v>
+        <v>0.7145</v>
       </c>
       <c r="N68" s="9" t="n">
-        <v>0.7112000000000001</v>
+        <v>0.7254</v>
       </c>
     </row>
     <row r="69">
@@ -4092,31 +4092,31 @@
         <v>4</v>
       </c>
       <c r="F69" t="n">
-        <v>0.0958</v>
+        <v>0.0752</v>
       </c>
       <c r="G69" t="n">
-        <v>0.0818</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="H69" s="9" t="n">
-        <v>0.0882</v>
+        <v>0.0762</v>
       </c>
       <c r="I69" t="n">
-        <v>0.2589</v>
+        <v>0.1533</v>
       </c>
       <c r="J69" t="n">
-        <v>0.2189</v>
+        <v>0.1325</v>
       </c>
       <c r="K69" s="9" t="n">
-        <v>0.2372</v>
+        <v>0.1421</v>
       </c>
       <c r="L69" t="n">
-        <v>0.7625999999999999</v>
+        <v>0.7287</v>
       </c>
       <c r="M69" t="n">
-        <v>0.7584</v>
+        <v>0.7146</v>
       </c>
       <c r="N69" s="9" t="n">
-        <v>0.7605</v>
+        <v>0.7216</v>
       </c>
     </row>
     <row r="70">
@@ -4204,19 +4204,19 @@
         <v>0.3003</v>
       </c>
       <c r="J71" t="n">
-        <v>0.2148</v>
+        <v>0.2113</v>
       </c>
       <c r="K71" s="9" t="n">
-        <v>0.2504</v>
+        <v>0.248</v>
       </c>
       <c r="L71" t="n">
         <v>0.7248</v>
       </c>
       <c r="M71" t="n">
-        <v>0.7266</v>
+        <v>0.7235</v>
       </c>
       <c r="N71" s="9" t="n">
-        <v>0.7257</v>
+        <v>0.7241</v>
       </c>
     </row>
     <row r="72">
@@ -4395,28 +4395,28 @@
         <v>0.0914</v>
       </c>
       <c r="G75" t="n">
-        <v>0.0623</v>
+        <v>0.0804</v>
       </c>
       <c r="H75" s="9" t="n">
-        <v>0.0741</v>
+        <v>0.08550000000000001</v>
       </c>
       <c r="I75" t="n">
         <v>0.1792</v>
       </c>
       <c r="J75" t="n">
-        <v>0.1381</v>
+        <v>0.1391</v>
       </c>
       <c r="K75" s="9" t="n">
-        <v>0.156</v>
+        <v>0.1566</v>
       </c>
       <c r="L75" t="n">
         <v>0.7853</v>
       </c>
       <c r="M75" t="n">
-        <v>0.7688</v>
+        <v>0.7649</v>
       </c>
       <c r="N75" s="9" t="n">
-        <v>0.777</v>
+        <v>0.775</v>
       </c>
     </row>
     <row r="76">
@@ -4442,31 +4442,31 @@
         <v>4</v>
       </c>
       <c r="F76" t="n">
-        <v>0.1562</v>
+        <v>0.1521</v>
       </c>
       <c r="G76" t="n">
-        <v>0.1025</v>
+        <v>0.1087</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>0.1237</v>
+        <v>0.1268</v>
       </c>
       <c r="I76" t="n">
-        <v>0.2962</v>
+        <v>0.3014</v>
       </c>
       <c r="J76" t="n">
-        <v>0.2528</v>
+        <v>0.2456</v>
       </c>
       <c r="K76" s="9" t="n">
-        <v>0.2727</v>
+        <v>0.2707</v>
       </c>
       <c r="L76" t="n">
-        <v>0.7989000000000001</v>
+        <v>0.7618</v>
       </c>
       <c r="M76" t="n">
-        <v>0.7625999999999999</v>
+        <v>0.7377</v>
       </c>
       <c r="N76" s="9" t="n">
-        <v>0.7803</v>
+        <v>0.7496</v>
       </c>
     </row>
     <row r="77">
@@ -4536,37 +4536,37 @@
         </is>
       </c>
       <c r="D78" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E78" s="8" t="n">
         <v>4</v>
       </c>
       <c r="F78" t="n">
-        <v>0.0112</v>
+        <v>0.0541</v>
       </c>
       <c r="G78" t="n">
-        <v>0.0064</v>
+        <v>0.0581</v>
       </c>
       <c r="H78" s="9" t="n">
-        <v>0.0081</v>
+        <v>0.056</v>
       </c>
       <c r="I78" t="n">
-        <v>0.1689</v>
+        <v>0.1825</v>
       </c>
       <c r="J78" t="n">
-        <v>0.0955</v>
+        <v>0.1656</v>
       </c>
       <c r="K78" s="9" t="n">
-        <v>0.122</v>
+        <v>0.1736</v>
       </c>
       <c r="L78" t="n">
-        <v>0.7248</v>
+        <v>0.7641</v>
       </c>
       <c r="M78" t="n">
-        <v>0.7095</v>
+        <v>0.7653</v>
       </c>
       <c r="N78" s="9" t="n">
-        <v>0.7171</v>
+        <v>0.7647</v>
       </c>
     </row>
     <row r="79">
@@ -4604,19 +4604,19 @@
         <v>0.1201</v>
       </c>
       <c r="J79" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.0989</v>
       </c>
       <c r="K79" s="9" t="n">
-        <v>0.1074</v>
+        <v>0.1085</v>
       </c>
       <c r="L79" t="n">
-        <v>0.735</v>
+        <v>0.7508</v>
       </c>
       <c r="M79" t="n">
-        <v>0.6945</v>
+        <v>0.7094</v>
       </c>
       <c r="N79" s="9" t="n">
-        <v>0.7141</v>
+        <v>0.7295</v>
       </c>
     </row>
     <row r="80">
@@ -4642,31 +4642,31 @@
         <v>4</v>
       </c>
       <c r="F80" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.08450000000000001</v>
       </c>
       <c r="G80" t="n">
-        <v>0.0704</v>
+        <v>0.0833</v>
       </c>
       <c r="H80" s="9" t="n">
-        <v>0.0732</v>
+        <v>0.0839</v>
       </c>
       <c r="I80" t="n">
-        <v>0.2166</v>
+        <v>0.2268</v>
       </c>
       <c r="J80" t="n">
-        <v>0.2006</v>
+        <v>0.2096</v>
       </c>
       <c r="K80" s="9" t="n">
-        <v>0.2083</v>
+        <v>0.2179</v>
       </c>
       <c r="L80" t="n">
-        <v>0.7634</v>
+        <v>0.7502</v>
       </c>
       <c r="M80" t="n">
-        <v>0.754</v>
+        <v>0.7395</v>
       </c>
       <c r="N80" s="9" t="n">
-        <v>0.7586000000000001</v>
+        <v>0.7449</v>
       </c>
     </row>
     <row r="81">
@@ -4710,13 +4710,13 @@
         <v>0.1958</v>
       </c>
       <c r="L81" t="n">
-        <v>0.7922</v>
+        <v>0.8008999999999999</v>
       </c>
       <c r="M81" t="n">
-        <v>0.7776999999999999</v>
+        <v>0.7941</v>
       </c>
       <c r="N81" s="9" t="n">
-        <v>0.7849</v>
+        <v>0.7975</v>
       </c>
     </row>
     <row r="82">

</xml_diff>